<commit_message>
results check and prep in ecxel
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/LNG_locations.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/LNG_locations.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28623"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3652ED6-DA3C-4FAB-AA19-AA9FC737C438}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Sheet1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -482,8 +488,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -526,50 +531,49 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:D80" displayName="Table1" name="Table1" id="1" totalsRowShown="0">
-  <autoFilter ref="A1:D80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:D80" totalsRowShown="0">
+  <autoFilter ref="A1:D80" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="4">
-    <tableColumn name="Country" id="1"/>
-    <tableColumn name="Name of _x000a_installation" id="2"/>
-    <tableColumn name="City" id="3"/>
-    <tableColumn name="Model Year" id="4"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Country"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name of _x000a_installation"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="City"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Model Year" dataDxfId="0"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showColumnStripes="0" showRowStripes="1" showLastColumn="0" showFirstColumn="0"/>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -578,10 +582,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -619,71 +623,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -711,7 +715,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -734,11 +738,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -747,13 +751,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -763,7 +767,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -772,7 +776,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -781,7 +785,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -789,10 +793,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -857,1619 +861,1617 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:F80"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" style="5" width="9.862142857142858" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="5" width="39.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="5" width="39.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="6" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="5" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="39.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="32.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="32.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="3">
-        <v>40.449271</v>
-      </c>
-      <c r="F2" s="3">
-        <v>19.480761</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="1" t="s">
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2">
+        <v>40.449271000000003</v>
+      </c>
+      <c r="F2" s="2">
+        <v>19.480761000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
       <c r="D3" s="4">
         <v>2021</v>
       </c>
-      <c r="E3" s="3">
-        <v>51.353</v>
-      </c>
-      <c r="F3" s="3">
+      <c r="E3" s="2">
+        <v>51.353000000000002</v>
+      </c>
+      <c r="F3" s="2">
         <v>3.22241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="4">
         <v>2024</v>
       </c>
-      <c r="E4" s="3">
-        <v>51.353</v>
-      </c>
-      <c r="F4" s="3">
+      <c r="E4" s="2">
+        <v>51.353000000000002</v>
+      </c>
+      <c r="F4" s="2">
         <v>3.22241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="4">
         <v>2035</v>
       </c>
-      <c r="E5" s="3">
-        <v>51.353</v>
-      </c>
-      <c r="F5" s="3">
+      <c r="E5" s="2">
+        <v>51.353000000000002</v>
+      </c>
+      <c r="F5" s="2">
         <v>3.22241</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>14</v>
       </c>
       <c r="D6" s="4">
         <v>2021</v>
       </c>
-      <c r="E6" s="3">
-        <v>45.211944</v>
-      </c>
-      <c r="F6" s="3">
+      <c r="E6" s="2">
+        <v>45.211944000000003</v>
+      </c>
+      <c r="F6" s="2">
         <v>14.554167</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="4">
         <v>2035</v>
       </c>
-      <c r="E7" s="3">
-        <v>45.211944</v>
-      </c>
-      <c r="F7" s="3">
+      <c r="E7" s="2">
+        <v>45.211944000000003</v>
+      </c>
+      <c r="F7" s="2">
         <v>14.554167</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="3">
-        <v>34.720244</v>
-      </c>
-      <c r="F8" s="3">
-        <v>33.32384</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="1" t="s">
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="2">
+        <v>34.720244000000001</v>
+      </c>
+      <c r="F8" s="2">
+        <v>33.323839999999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>19</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="3">
-        <v>29.64863</v>
-      </c>
-      <c r="F9" s="1" t="s">
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="2">
+        <v>29.648630000000001</v>
+      </c>
+      <c r="F9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="3">
-        <v>29.64863</v>
-      </c>
-      <c r="F10" s="1" t="s">
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="2">
+        <v>29.648630000000001</v>
+      </c>
+      <c r="F10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>24</v>
       </c>
       <c r="D11" s="4">
         <v>2035</v>
       </c>
-      <c r="E11" s="3">
-        <v>59.38445</v>
-      </c>
-      <c r="F11" s="3">
-        <v>24.07494</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75">
-      <c r="A12" s="1" t="s">
+      <c r="E11" s="2">
+        <v>59.384450000000001</v>
+      </c>
+      <c r="F11" s="2">
+        <v>24.074940000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="3">
-        <v>59.50601</v>
-      </c>
-      <c r="F12" s="3">
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="2">
+        <v>59.506010000000003</v>
+      </c>
+      <c r="F12" s="2">
         <v>25.0045</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>28</v>
       </c>
       <c r="D13" s="4">
         <v>2024</v>
       </c>
-      <c r="E13" s="3">
-        <v>60.013697</v>
-      </c>
-      <c r="F13" s="1" t="s">
+      <c r="E13" s="2">
+        <v>60.013697000000001</v>
+      </c>
+      <c r="F13" t="s">
         <v>29</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>32</v>
       </c>
       <c r="D14" s="4">
         <v>2021</v>
       </c>
-      <c r="E14" s="3">
-        <v>51.03361</v>
-      </c>
-      <c r="F14" s="3">
-        <v>2.19653</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75">
-      <c r="A15" s="1" t="s">
+      <c r="E14" s="2">
+        <v>51.033610000000003</v>
+      </c>
+      <c r="F14" s="2">
+        <v>2.1965300000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>34</v>
       </c>
       <c r="D15" s="4">
         <v>2021</v>
       </c>
-      <c r="E15" s="3">
-        <v>43.41963</v>
-      </c>
-      <c r="F15" s="3">
-        <v>4.90102</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75">
-      <c r="A16" s="1" t="s">
+      <c r="E15" s="2">
+        <v>43.419629999999998</v>
+      </c>
+      <c r="F15" s="2">
+        <v>4.9010199999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>34</v>
       </c>
       <c r="D16" s="4">
         <v>2024</v>
       </c>
-      <c r="E16" s="3">
-        <v>43.41963</v>
-      </c>
-      <c r="F16" s="3">
-        <v>4.90102</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75">
-      <c r="A17" s="1" t="s">
+      <c r="E16" s="2">
+        <v>43.419629999999998</v>
+      </c>
+      <c r="F16" s="2">
+        <v>4.9010199999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>34</v>
       </c>
       <c r="D17" s="4">
         <v>2035</v>
       </c>
-      <c r="E17" s="3">
-        <v>43.41963</v>
-      </c>
-      <c r="F17" s="3">
-        <v>4.90102</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75">
-      <c r="A18" s="1" t="s">
+      <c r="E17" s="2">
+        <v>43.419629999999998</v>
+      </c>
+      <c r="F17" s="2">
+        <v>4.9010199999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>34</v>
       </c>
       <c r="D18" s="4">
         <v>2021</v>
       </c>
-      <c r="E18" s="3">
-        <v>43.454</v>
-      </c>
-      <c r="F18" s="3">
-        <v>4.85167</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75">
-      <c r="A19" s="1" t="s">
+      <c r="E18" s="2">
+        <v>43.454000000000001</v>
+      </c>
+      <c r="F18" s="2">
+        <v>4.8516700000000004</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>37</v>
       </c>
       <c r="D19" s="4">
         <v>2021</v>
       </c>
-      <c r="E19" s="3">
-        <v>47.30296</v>
-      </c>
-      <c r="F19" s="3">
-        <v>-2.14278</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75">
-      <c r="A20" s="1" t="s">
+      <c r="E19" s="2">
+        <v>47.302959999999999</v>
+      </c>
+      <c r="F19" s="2">
+        <v>-2.1427800000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>30</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>39</v>
       </c>
       <c r="D20" s="4">
         <v>2024</v>
       </c>
-      <c r="E20" s="3">
-        <v>49.475</v>
-      </c>
-      <c r="F20" s="3">
-        <v>0.133333</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75">
-      <c r="A21" s="1" t="s">
+      <c r="E20" s="2">
+        <v>49.475000000000001</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0.13333300000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
         <v>42</v>
       </c>
       <c r="D21" s="4">
         <v>2024</v>
       </c>
-      <c r="E21" s="3">
-        <v>53.9140009</v>
-      </c>
-      <c r="F21" s="3">
-        <v>8.9760945</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75">
-      <c r="A22" s="1" t="s">
+      <c r="E21" s="2">
+        <v>53.914000899999998</v>
+      </c>
+      <c r="F21" s="2">
+        <v>8.9760945000000003</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>40</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" t="s">
         <v>44</v>
       </c>
       <c r="D22" s="4">
         <v>2024</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="2">
         <v>53.652459</v>
       </c>
-      <c r="F22" s="3">
-        <v>9.510382</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75">
-      <c r="A23" s="1" t="s">
+      <c r="F22" s="2">
+        <v>9.5103819999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>40</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" t="s">
         <v>46</v>
       </c>
       <c r="D23" s="4">
         <v>2024</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="2">
         <v>53.6417</v>
       </c>
-      <c r="F23" s="3">
-        <v>8.1089</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75">
-      <c r="A24" s="1" t="s">
+      <c r="F23" s="2">
+        <v>8.1089000000000002</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" t="s">
         <v>46</v>
       </c>
       <c r="D24" s="4">
         <v>2024</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="2">
         <v>53.6417</v>
       </c>
-      <c r="F24" s="3">
-        <v>8.1089</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75">
-      <c r="A25" s="1" t="s">
+      <c r="F24" s="2">
+        <v>8.1089000000000002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E25" s="3">
-        <v>54.153332</v>
-      </c>
-      <c r="F25" s="3">
-        <v>13.645319</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75">
-      <c r="A26" s="1" t="s">
+      <c r="C25" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="2">
+        <v>54.153331999999999</v>
+      </c>
+      <c r="F25" s="2">
+        <v>13.645319000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>49</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" t="s">
         <v>50</v>
       </c>
       <c r="D26" s="4">
         <v>2024</v>
       </c>
-      <c r="E26" s="3">
-        <v>54.478384</v>
-      </c>
-      <c r="F26" s="3">
-        <v>13.598351</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75">
-      <c r="A27" s="1" t="s">
+      <c r="E26" s="2">
+        <v>54.478383999999998</v>
+      </c>
+      <c r="F26" s="2">
+        <v>13.598350999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>51</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" t="s">
         <v>50</v>
       </c>
       <c r="D27" s="4">
         <v>2024</v>
       </c>
-      <c r="E27" s="3">
-        <v>54.478384</v>
-      </c>
-      <c r="F27" s="3">
-        <v>13.598351</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75">
-      <c r="A28" s="1" t="s">
+      <c r="E27" s="2">
+        <v>54.478383999999998</v>
+      </c>
+      <c r="F27" s="2">
+        <v>13.598350999999999</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>46</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" t="s">
         <v>46</v>
       </c>
       <c r="D28" s="4">
         <v>2035</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28" s="2">
         <v>53.6417</v>
       </c>
-      <c r="F28" s="3">
-        <v>8.1089</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75">
-      <c r="A29" s="1" t="s">
+      <c r="F28" s="2">
+        <v>8.1089000000000002</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" t="s">
         <v>44</v>
       </c>
       <c r="D29" s="4">
         <v>2035</v>
       </c>
-      <c r="E29" s="3">
+      <c r="E29" s="2">
         <v>53.652459</v>
       </c>
-      <c r="F29" s="3">
-        <v>9.510382</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75">
-      <c r="A30" s="1" t="s">
+      <c r="F29" s="2">
+        <v>9.5103819999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>54</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E30" s="3">
-        <v>37.91092</v>
-      </c>
-      <c r="F30" s="3">
-        <v>23.063539</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75">
-      <c r="A31" s="1" t="s">
+      <c r="C30" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E30" s="2">
+        <v>37.910919999999997</v>
+      </c>
+      <c r="F30" s="2">
+        <v>23.063538999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>55</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" t="s">
         <v>56</v>
       </c>
       <c r="D31" s="4">
         <v>2024</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31" s="2">
         <v>40.84995</v>
       </c>
-      <c r="F31" s="3">
-        <v>25.87644</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75">
-      <c r="A32" s="1" t="s">
+      <c r="F31" s="2">
+        <v>25.876439999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>57</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E32" s="3">
-        <v>40.748354</v>
-      </c>
-      <c r="F32" s="3">
-        <v>25.718754</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75">
-      <c r="A33" s="1" t="s">
+      <c r="C32" t="s">
+        <v>8</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E32" s="2">
+        <v>40.748353999999999</v>
+      </c>
+      <c r="F32" s="2">
+        <v>25.718754000000001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>53</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>58</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" t="s">
         <v>59</v>
       </c>
       <c r="D33" s="4">
         <v>2021</v>
       </c>
-      <c r="E33" s="3">
+      <c r="E33" s="2">
         <v>37.96</v>
       </c>
-      <c r="F33" s="3">
+      <c r="F33" s="2">
         <v>23.4023</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
-      <c r="A34" s="1" t="s">
+    <row r="34" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>53</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>60</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" t="s">
         <v>61</v>
       </c>
       <c r="D34" s="4">
         <v>2024</v>
       </c>
-      <c r="E34" s="3">
-        <v>39.3512644</v>
-      </c>
-      <c r="F34" s="3">
-        <v>22.9324904</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75">
-      <c r="A35" s="1" t="s">
+      <c r="E34" s="2">
+        <v>39.351264399999998</v>
+      </c>
+      <c r="F34" s="2">
+        <v>22.932490399999999</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>53</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>62</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" t="s">
         <v>63</v>
       </c>
       <c r="D35" s="4">
         <v>2035</v>
       </c>
-      <c r="E35" s="3">
-        <v>40.2893</v>
-      </c>
-      <c r="F35" s="3">
-        <v>23.025</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75">
-      <c r="A36" s="1" t="s">
+      <c r="E35" s="2">
+        <v>40.289299999999997</v>
+      </c>
+      <c r="F35" s="2">
+        <v>23.024999999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>64</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" t="s">
         <v>65</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" s="3">
+      <c r="C36" t="s">
+        <v>8</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" s="2">
         <v>52.58099</v>
       </c>
-      <c r="F36" s="3">
-        <v>-9.44246</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75">
-      <c r="A37" s="1" t="s">
+      <c r="F36" s="2">
+        <v>-9.4424600000000005</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>64</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" t="s">
         <v>66</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" t="s">
         <v>67</v>
       </c>
       <c r="D37" s="4">
         <v>2035</v>
       </c>
-      <c r="E37" s="3">
+      <c r="E37" s="2">
         <v>51.264274</v>
       </c>
-      <c r="F37" s="3">
-        <v>-8.045619</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75">
-      <c r="A38" s="1" t="s">
+      <c r="F37" s="2">
+        <v>-8.0456190000000003</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>69</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E38" s="3">
-        <v>32.45</v>
-      </c>
-      <c r="F38" s="3">
-        <v>34.916667</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75">
-      <c r="A39" s="1" t="s">
+      <c r="C38" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" s="2">
+        <v>32.450000000000003</v>
+      </c>
+      <c r="F38" s="2">
+        <v>34.916666999999997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>70</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>71</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" t="s">
         <v>72</v>
       </c>
       <c r="D39" s="4">
         <v>2021</v>
       </c>
-      <c r="E39" s="3">
+      <c r="E39" s="2">
         <v>43.644444</v>
       </c>
-      <c r="F39" s="3">
-        <v>9.988889</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75">
-      <c r="A40" s="1" t="s">
+      <c r="F39" s="2">
+        <v>9.9888890000000004</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>70</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" t="s">
         <v>73</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" t="s">
         <v>74</v>
       </c>
       <c r="D40" s="4">
         <v>2021</v>
       </c>
-      <c r="E40" s="3">
-        <v>44.07428</v>
-      </c>
-      <c r="F40" s="3">
-        <v>9.83087</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75">
-      <c r="A41" s="1" t="s">
+      <c r="E40" s="2">
+        <v>44.074280000000002</v>
+      </c>
+      <c r="F40" s="2">
+        <v>9.8308700000000009</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>70</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" t="s">
         <v>75</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" t="s">
         <v>76</v>
       </c>
       <c r="D41" s="4">
         <v>2024</v>
       </c>
-      <c r="E41" s="3">
-        <v>42.932151</v>
-      </c>
-      <c r="F41" s="3">
+      <c r="E41" s="2">
+        <v>42.932150999999998</v>
+      </c>
+      <c r="F41" s="2">
         <v>10.54641</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75">
-      <c r="A42" s="1" t="s">
+    <row r="42" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>70</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" t="s">
         <v>77</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" t="s">
         <v>78</v>
       </c>
       <c r="D42" s="4">
         <v>2024</v>
       </c>
-      <c r="E42" s="3">
+      <c r="E42" s="2">
         <v>44.48283</v>
       </c>
-      <c r="F42" s="3">
+      <c r="F42" s="2">
         <v>12.291482</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75">
-      <c r="A43" s="1" t="s">
+    <row r="43" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>70</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" t="s">
         <v>79</v>
       </c>
-      <c r="C43" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E43" s="3">
-        <v>37.28297</v>
-      </c>
-      <c r="F43" s="3">
-        <v>13.53774</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75">
-      <c r="A44" s="1" t="s">
+      <c r="C43" t="s">
+        <v>8</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E43" s="2">
+        <v>37.282969999999999</v>
+      </c>
+      <c r="F43" s="2">
+        <v>13.537739999999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>70</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" t="s">
         <v>80</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C44" t="s">
         <v>81</v>
       </c>
       <c r="D44" s="4">
         <v>2021</v>
       </c>
-      <c r="E44" s="3">
-        <v>45.091667</v>
-      </c>
-      <c r="F44" s="3">
-        <v>12.586111</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75">
-      <c r="A45" s="1" t="s">
+      <c r="E44" s="2">
+        <v>45.091667000000001</v>
+      </c>
+      <c r="F44" s="2">
+        <v>12.586111000000001</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>82</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" t="s">
         <v>83</v>
       </c>
-      <c r="C45" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E45" s="3">
-        <v>57.315</v>
-      </c>
-      <c r="F45" s="3">
-        <v>24.367</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75">
-      <c r="A46" s="1" t="s">
+      <c r="C45" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E45" s="2">
+        <v>57.314999999999998</v>
+      </c>
+      <c r="F45" s="2">
+        <v>24.367000000000001</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>84</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" t="s">
         <v>85</v>
       </c>
-      <c r="C46" s="1" t="s">
+      <c r="C46" t="s">
         <v>86</v>
       </c>
       <c r="D46" s="4">
         <v>2021</v>
       </c>
-      <c r="E46" s="3">
+      <c r="E46" s="2">
         <v>55.66451</v>
       </c>
-      <c r="F46" s="3">
-        <v>21.13762</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75">
-      <c r="A47" s="1" t="s">
+      <c r="F46" s="2">
+        <v>21.137619999999998</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>87</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" t="s">
         <v>88</v>
       </c>
-      <c r="C47" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E47" s="3">
+      <c r="C47" t="s">
+        <v>8</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E47" s="2">
         <v>35.8277</v>
       </c>
-      <c r="F47" s="3">
+      <c r="F47" s="2">
         <v>14.5542</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75">
-      <c r="A48" s="1" t="s">
+    <row r="48" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>89</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>90</v>
       </c>
-      <c r="C48" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E48" s="3">
+      <c r="C48" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E48" s="2">
         <v>33.1267</v>
       </c>
-      <c r="F48" s="3">
-        <v>-8.62028</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75">
-      <c r="A49" s="1" t="s">
+      <c r="F48" s="2">
+        <v>-8.6202799999999993</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>89</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" t="s">
         <v>91</v>
       </c>
-      <c r="C49" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E49" s="3">
-        <v>33.71339</v>
-      </c>
-      <c r="F49" s="1" t="s">
+      <c r="C49" t="s">
+        <v>8</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E49" s="2">
+        <v>33.713389999999997</v>
+      </c>
+      <c r="F49" t="s">
         <v>92</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75">
-      <c r="A50" s="1" t="s">
+    <row r="50" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>93</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" t="s">
         <v>94</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C50" t="s">
         <v>95</v>
       </c>
       <c r="D50" s="4">
         <v>2021</v>
       </c>
-      <c r="E50" s="3">
-        <v>51.971111</v>
-      </c>
-      <c r="F50" s="3">
-        <v>4.068889</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75">
-      <c r="A51" s="1" t="s">
+      <c r="E50" s="2">
+        <v>51.971111000000001</v>
+      </c>
+      <c r="F50" s="2">
+        <v>4.0688890000000004</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>93</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" t="s">
         <v>94</v>
       </c>
-      <c r="C51" s="1" t="s">
+      <c r="C51" t="s">
         <v>95</v>
       </c>
       <c r="D51" s="4">
         <v>2024</v>
       </c>
-      <c r="E51" s="3">
-        <v>51.971111</v>
-      </c>
-      <c r="F51" s="3">
-        <v>4.068889</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75">
-      <c r="A52" s="1" t="s">
+      <c r="E51" s="2">
+        <v>51.971111000000001</v>
+      </c>
+      <c r="F51" s="2">
+        <v>4.0688890000000004</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>93</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" t="s">
         <v>94</v>
       </c>
-      <c r="C52" s="1" t="s">
+      <c r="C52" t="s">
         <v>95</v>
       </c>
       <c r="D52" s="4">
         <v>2035</v>
       </c>
-      <c r="E52" s="3">
-        <v>51.971111</v>
-      </c>
-      <c r="F52" s="3">
-        <v>4.068889</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75">
-      <c r="A53" s="1" t="s">
+      <c r="E52" s="2">
+        <v>51.971111000000001</v>
+      </c>
+      <c r="F52" s="2">
+        <v>4.0688890000000004</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>93</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" t="s">
         <v>96</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C53" t="s">
         <v>97</v>
       </c>
       <c r="D53" s="4">
         <v>2024</v>
       </c>
-      <c r="E53" s="3">
-        <v>53.4356487</v>
-      </c>
-      <c r="F53" s="3">
-        <v>6.8330977</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75">
-      <c r="A54" s="1" t="s">
+      <c r="E53" s="2">
+        <v>53.435648700000002</v>
+      </c>
+      <c r="F53" s="2">
+        <v>6.8330976999999997</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>98</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" t="s">
         <v>99</v>
       </c>
-      <c r="C54" s="1" t="s">
+      <c r="C54" t="s">
         <v>100</v>
       </c>
       <c r="D54" s="4">
         <v>2035</v>
       </c>
-      <c r="E54" s="3">
-        <v>54.424696</v>
-      </c>
-      <c r="F54" s="3">
-        <v>18.73585</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75">
-      <c r="A55" s="1" t="s">
+      <c r="E54" s="2">
+        <v>54.424695999999997</v>
+      </c>
+      <c r="F54" s="2">
+        <v>18.735849999999999</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>98</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" t="s">
         <v>101</v>
       </c>
-      <c r="C55" s="1" t="s">
+      <c r="C55" t="s">
         <v>102</v>
       </c>
       <c r="D55" s="4">
         <v>2021</v>
       </c>
-      <c r="E55" s="3">
-        <v>53.909167</v>
-      </c>
-      <c r="F55" s="3">
+      <c r="E55" s="2">
+        <v>53.909166999999997</v>
+      </c>
+      <c r="F55" s="2">
         <v>14.294722</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75">
-      <c r="A56" s="1" t="s">
+    <row r="56" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>98</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" t="s">
         <v>101</v>
       </c>
-      <c r="C56" s="1" t="s">
+      <c r="C56" t="s">
         <v>102</v>
       </c>
       <c r="D56" s="4">
         <v>2024</v>
       </c>
-      <c r="E56" s="3">
-        <v>53.909167</v>
-      </c>
-      <c r="F56" s="3">
+      <c r="E56" s="2">
+        <v>53.909166999999997</v>
+      </c>
+      <c r="F56" s="2">
         <v>14.294722</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75">
-      <c r="A57" s="1" t="s">
+    <row r="57" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>103</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" t="s">
         <v>104</v>
       </c>
-      <c r="C57" s="1" t="s">
+      <c r="C57" t="s">
         <v>105</v>
       </c>
       <c r="D57" s="4">
         <v>2021</v>
       </c>
-      <c r="E57" s="3">
-        <v>37.9419</v>
-      </c>
-      <c r="F57" s="1" t="s">
+      <c r="E57" s="2">
+        <v>37.941899999999997</v>
+      </c>
+      <c r="F57" t="s">
         <v>106</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75">
-      <c r="A58" s="1" t="s">
+    <row r="58" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>107</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" t="s">
         <v>108</v>
       </c>
-      <c r="C58" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E58" s="3">
+      <c r="C58" t="s">
+        <v>8</v>
+      </c>
+      <c r="D58" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E58" s="2">
         <v>55.017806</v>
       </c>
-      <c r="F58" s="3">
-        <v>20.323333</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75">
-      <c r="A59" s="1" t="s">
+      <c r="F58" s="2">
+        <v>20.323333000000002</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>109</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" t="s">
         <v>110</v>
       </c>
-      <c r="C59" s="1" t="s">
+      <c r="C59" t="s">
         <v>111</v>
       </c>
       <c r="D59" s="4">
         <v>2021</v>
       </c>
-      <c r="E59" s="3">
-        <v>41.3394</v>
-      </c>
-      <c r="F59" s="3">
-        <v>2.1583</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75">
-      <c r="A60" s="1" t="s">
+      <c r="E59" s="2">
+        <v>41.339399999999998</v>
+      </c>
+      <c r="F59" s="2">
+        <v>2.1583000000000001</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>109</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" t="s">
         <v>112</v>
       </c>
-      <c r="C60" s="1" t="s">
+      <c r="C60" t="s">
         <v>113</v>
       </c>
       <c r="D60" s="4">
         <v>2021</v>
       </c>
-      <c r="E60" s="1" t="s">
+      <c r="E60" t="s">
         <v>114</v>
       </c>
-      <c r="F60" s="3">
-        <v>-3.09473</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75">
-      <c r="A61" s="1" t="s">
+      <c r="F60" s="2">
+        <v>-3.0947300000000002</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>109</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" t="s">
         <v>115</v>
       </c>
-      <c r="C61" s="1" t="s">
+      <c r="C61" t="s">
         <v>116</v>
       </c>
       <c r="D61" s="4">
         <v>2021</v>
       </c>
-      <c r="E61" s="3">
-        <v>37.57457</v>
-      </c>
-      <c r="F61" s="3">
-        <v>-0.9595</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75">
-      <c r="A62" s="1" t="s">
+      <c r="E61" s="2">
+        <v>37.574570000000001</v>
+      </c>
+      <c r="F61" s="2">
+        <v>-0.95950000000000002</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>109</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B62" t="s">
         <v>117</v>
       </c>
-      <c r="C62" s="1" t="s">
+      <c r="C62" t="s">
         <v>118</v>
       </c>
       <c r="D62" s="4">
         <v>2024</v>
       </c>
-      <c r="E62" s="3">
-        <v>43.5696</v>
-      </c>
-      <c r="F62" s="3">
-        <v>-5.6934</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75">
-      <c r="A63" s="1" t="s">
+      <c r="E62" s="2">
+        <v>43.569600000000001</v>
+      </c>
+      <c r="F62" s="2">
+        <v>-5.6933999999999996</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>109</v>
       </c>
-      <c r="B63" s="1" t="s">
+      <c r="B63" t="s">
         <v>119</v>
       </c>
-      <c r="C63" s="1" t="s">
+      <c r="C63" t="s">
         <v>120</v>
       </c>
       <c r="D63" s="4">
         <v>2021</v>
       </c>
-      <c r="E63" s="3">
-        <v>37.17355</v>
-      </c>
-      <c r="F63" s="3">
-        <v>-6.911</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75">
-      <c r="A64" s="1" t="s">
+      <c r="E63" s="2">
+        <v>37.173549999999999</v>
+      </c>
+      <c r="F63" s="2">
+        <v>-6.9109999999999996</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>109</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B64" t="s">
         <v>121</v>
       </c>
-      <c r="C64" s="1" t="s">
+      <c r="C64" t="s">
         <v>122</v>
       </c>
       <c r="D64" s="4">
         <v>2021</v>
       </c>
-      <c r="E64" s="3">
-        <v>43.4613</v>
-      </c>
-      <c r="F64" s="3">
-        <v>-8.2395</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75">
-      <c r="A65" s="1" t="s">
+      <c r="E64" s="2">
+        <v>43.461300000000001</v>
+      </c>
+      <c r="F64" s="2">
+        <v>-8.2394999999999996</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>109</v>
       </c>
-      <c r="B65" s="1" t="s">
+      <c r="B65" t="s">
         <v>123</v>
       </c>
-      <c r="C65" s="1" t="s">
+      <c r="C65" t="s">
         <v>124</v>
       </c>
       <c r="D65" s="4">
         <v>2021</v>
       </c>
-      <c r="E65" s="3">
-        <v>39.6329</v>
-      </c>
-      <c r="F65" s="3">
+      <c r="E65" s="2">
+        <v>39.632899999999999</v>
+      </c>
+      <c r="F65" s="2">
         <v>-0.2152</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75">
-      <c r="A66" s="1" t="s">
+    <row r="66" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>125</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B66" t="s">
         <v>126</v>
       </c>
-      <c r="C66" s="1" t="s">
+      <c r="C66" t="s">
         <v>126</v>
       </c>
       <c r="D66" s="4">
         <v>2021</v>
       </c>
-      <c r="E66" s="3">
-        <v>38.74443</v>
-      </c>
-      <c r="F66" s="3">
-        <v>26.895665</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75">
-      <c r="A67" s="1" t="s">
+      <c r="E66" s="2">
+        <v>38.744430000000001</v>
+      </c>
+      <c r="F66" s="2">
+        <v>26.895665000000001</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>125</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B67" t="s">
         <v>127</v>
       </c>
-      <c r="C67" s="1" t="s">
+      <c r="C67" t="s">
         <v>128</v>
       </c>
       <c r="D67" s="4">
         <v>2021</v>
       </c>
-      <c r="E67" s="3">
-        <v>38.82245489</v>
-      </c>
-      <c r="F67" s="3">
-        <v>26.91411088</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75">
-      <c r="A68" s="1" t="s">
+      <c r="E67" s="2">
+        <v>38.822454890000003</v>
+      </c>
+      <c r="F67" s="2">
+        <v>26.914110879999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>125</v>
       </c>
-      <c r="B68" s="1" t="s">
+      <c r="B68" t="s">
         <v>129</v>
       </c>
-      <c r="C68" s="1" t="s">
+      <c r="C68" t="s">
         <v>130</v>
       </c>
       <c r="D68" s="4">
         <v>2024</v>
       </c>
-      <c r="E68" s="3">
+      <c r="E68" s="2">
         <v>40.636702</v>
       </c>
-      <c r="F68" s="3">
-        <v>26.657427</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75">
-      <c r="A69" s="1" t="s">
+      <c r="F68" s="2">
+        <v>26.657426999999998</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>125</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B69" t="s">
         <v>131</v>
       </c>
-      <c r="C69" s="1" t="s">
+      <c r="C69" t="s">
         <v>132</v>
       </c>
       <c r="D69" s="4">
         <v>2021</v>
       </c>
-      <c r="E69" s="3">
-        <v>36.85099026</v>
-      </c>
-      <c r="F69" s="3">
-        <v>36.12597587</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75">
-      <c r="A70" s="1" t="s">
+      <c r="E69" s="2">
+        <v>36.850990260000003</v>
+      </c>
+      <c r="F69" s="2">
+        <v>36.125975869999998</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>125</v>
       </c>
-      <c r="B70" s="1" t="s">
+      <c r="B70" t="s">
         <v>133</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="C70" t="s">
         <v>134</v>
       </c>
       <c r="D70" s="4">
         <v>2021</v>
       </c>
-      <c r="E70" s="3">
-        <v>40.99201724</v>
-      </c>
-      <c r="F70" s="3">
-        <v>27.98607026</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75">
-      <c r="A71" s="1" t="s">
+      <c r="E70" s="2">
+        <v>40.992017240000003</v>
+      </c>
+      <c r="F70" s="2">
+        <v>27.986070260000002</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>135</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B71" t="s">
         <v>136</v>
       </c>
-      <c r="C71" s="1" t="s">
+      <c r="C71" t="s">
         <v>137</v>
       </c>
       <c r="D71" s="4">
         <v>2021</v>
       </c>
-      <c r="E71" s="3">
-        <v>51.45107</v>
-      </c>
-      <c r="F71" s="3">
-        <v>0.67987</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75">
-      <c r="A72" s="1" t="s">
+      <c r="E71" s="2">
+        <v>51.451070000000001</v>
+      </c>
+      <c r="F71" s="2">
+        <v>0.67986999999999997</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>135</v>
       </c>
-      <c r="B72" s="1" t="s">
+      <c r="B72" t="s">
         <v>136</v>
       </c>
-      <c r="C72" s="1" t="s">
+      <c r="C72" t="s">
         <v>137</v>
       </c>
       <c r="D72" s="4">
         <v>2035</v>
       </c>
-      <c r="E72" s="3">
-        <v>51.45107</v>
-      </c>
-      <c r="F72" s="3">
-        <v>0.67987</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75">
-      <c r="A73" s="1" t="s">
+      <c r="E72" s="2">
+        <v>51.451070000000001</v>
+      </c>
+      <c r="F72" s="2">
+        <v>0.67986999999999997</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>135</v>
       </c>
-      <c r="B73" s="1" t="s">
+      <c r="B73" t="s">
         <v>138</v>
       </c>
-      <c r="C73" s="1" t="s">
+      <c r="C73" t="s">
         <v>139</v>
       </c>
       <c r="D73" s="4">
         <v>2021</v>
       </c>
-      <c r="E73" s="3">
-        <v>51.70453</v>
-      </c>
-      <c r="F73" s="3">
-        <v>-4.99774</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75">
-      <c r="A74" s="1" t="s">
+      <c r="E73" s="2">
+        <v>51.704529999999998</v>
+      </c>
+      <c r="F73" s="2">
+        <v>-4.9977400000000003</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>135</v>
       </c>
-      <c r="B74" s="1" t="s">
+      <c r="B74" t="s">
         <v>140</v>
       </c>
-      <c r="C74" s="1" t="s">
+      <c r="C74" t="s">
         <v>139</v>
       </c>
       <c r="D74" s="4">
         <v>2021</v>
       </c>
-      <c r="E74" s="3">
-        <v>51.70453</v>
-      </c>
-      <c r="F74" s="3">
-        <v>-4.99774</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75">
-      <c r="A75" s="1" t="s">
+      <c r="E74" s="2">
+        <v>51.704529999999998</v>
+      </c>
+      <c r="F74" s="2">
+        <v>-4.9977400000000003</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>135</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B75" t="s">
         <v>141</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C75" t="s">
         <v>142</v>
       </c>
       <c r="D75" s="4">
         <v>2021</v>
       </c>
-      <c r="E75" s="3">
+      <c r="E75" s="2">
         <v>54.57423</v>
       </c>
-      <c r="F75" s="3">
-        <v>-1.23496</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75">
-      <c r="A76" s="1" t="s">
+      <c r="F75" s="2">
+        <v>-1.2349600000000001</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>143</v>
       </c>
-      <c r="B76" s="1" t="s">
+      <c r="B76" t="s">
         <v>144</v>
       </c>
-      <c r="C76" s="1" t="s">
+      <c r="C76" t="s">
         <v>145</v>
       </c>
       <c r="D76" s="4">
         <v>2021</v>
       </c>
-      <c r="E76" s="3">
-        <v>70.6854</v>
-      </c>
-      <c r="F76" s="3">
+      <c r="E76" s="2">
+        <v>70.685400000000001</v>
+      </c>
+      <c r="F76" s="2">
         <v>23.59</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75">
-      <c r="A77" s="1" t="s">
+    <row r="77" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>143</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B77" t="s">
         <v>146</v>
       </c>
-      <c r="C77" s="1" t="s">
+      <c r="C77" t="s">
         <v>147</v>
       </c>
       <c r="D77" s="4">
         <v>2021</v>
       </c>
-      <c r="E77" s="3">
-        <v>59.313521</v>
-      </c>
-      <c r="F77" s="1" t="s">
+      <c r="E77" s="2">
+        <v>59.313521000000001</v>
+      </c>
+      <c r="F77" t="s">
         <v>148</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75">
-      <c r="A78" s="1" t="s">
+    <row r="78" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>143</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B78" t="s">
         <v>149</v>
       </c>
-      <c r="C78" s="1" t="s">
+      <c r="C78" t="s">
         <v>150</v>
       </c>
       <c r="D78" s="4">
         <v>2021</v>
       </c>
-      <c r="E78" s="3">
-        <v>60.548447</v>
-      </c>
-      <c r="F78" s="3">
-        <v>4.834402</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75">
-      <c r="A79" s="1" t="s">
+      <c r="E78" s="2">
+        <v>60.548447000000003</v>
+      </c>
+      <c r="F78" s="2">
+        <v>4.8344019999999999</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>143</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="B79" t="s">
         <v>151</v>
       </c>
-      <c r="C79" s="1" t="s">
+      <c r="C79" t="s">
         <v>150</v>
       </c>
       <c r="D79" s="4">
         <v>2021</v>
       </c>
-      <c r="E79" s="3">
-        <v>60.548447</v>
-      </c>
-      <c r="F79" s="3">
-        <v>4.834402</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75">
-      <c r="A80" s="1" t="s">
+      <c r="E79" s="2">
+        <v>60.548447000000003</v>
+      </c>
+      <c r="F79" s="2">
+        <v>4.8344019999999999</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>143</v>
       </c>
-      <c r="B80" s="1" t="s">
+      <c r="B80" t="s">
         <v>152</v>
       </c>
-      <c r="C80" s="1" t="s">
+      <c r="C80" t="s">
         <v>153</v>
       </c>
       <c r="D80" s="4">
         <v>2021</v>
       </c>
-      <c r="E80" s="3">
-        <v>58.9237</v>
-      </c>
-      <c r="F80" s="3">
-        <v>5.5761</v>
+      <c r="E80" s="2">
+        <v>58.923699999999997</v>
+      </c>
+      <c r="F80" s="2">
+        <v>5.5761000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update LNG locations and add global terminals
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/LNG_locations.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/LNG_locations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6830430A-F7BE-4D8E-9365-DA76DD172B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACA48B3-2F51-43DA-8247-07333E081B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="195">
   <si>
     <t>Country</t>
   </si>
@@ -111,9 +111,6 @@
     <t>Ingå</t>
   </si>
   <si>
-    <t xml:space="preserve"> 23.91506</t>
-  </si>
-  <si>
     <t>France</t>
   </si>
   <si>
@@ -583,6 +580,33 @@
   </si>
   <si>
     <t>Vladivostok</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>Thailand</t>
+  </si>
+  <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>Qatar</t>
+  </si>
+  <si>
+    <t>Trinidad&amp;Tobago</t>
+  </si>
+  <si>
+    <t>UAE</t>
+  </si>
+  <si>
+    <t>Australia</t>
+  </si>
+  <si>
+    <t>ME</t>
+  </si>
+  <si>
+    <t>Asia</t>
   </si>
 </sst>
 </file>
@@ -647,7 +671,13 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -671,19 +701,21 @@
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Country"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Name of _x000a_installation"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="City"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Model Year" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Model Year" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BC26E397-192F-4143-ADEB-7D939A583460}" name="Table13" displayName="Table13" ref="A1:C24" totalsRowShown="0">
-  <autoFilter ref="A1:C24" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{BC26E397-192F-4143-ADEB-7D939A583460}" name="Table13" displayName="Table13" ref="A1:E24" totalsRowShown="0">
+  <autoFilter ref="A1:E24" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{0E3B5DB7-5434-46DF-BB52-FC4DF5B7FC64}" name="Country"/>
     <tableColumn id="2" xr3:uid="{829C8557-0003-40C1-8A7F-75D69F40D03A}" name="Region"/>
     <tableColumn id="3" xr3:uid="{4C01B8FA-327F-4B33-8672-F11DBA3FC23C}" name="City"/>
+    <tableColumn id="4" xr3:uid="{01EC782C-1A43-42C4-A033-218BDA60607B}" name="Latitude" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{7DFA174C-0888-4D1D-80F4-15B4443C64AC}" name="Longitude" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1162,7 +1194,7 @@
       <c r="E9" s="2">
         <v>29.648630000000001</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1182,7 +1214,7 @@
       <c r="E10" s="2">
         <v>29.648630000000001</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="2" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1242,19 +1274,19 @@
       <c r="E13" s="2">
         <v>60.013697000000001</v>
       </c>
-      <c r="F13" t="s">
-        <v>29</v>
+      <c r="F13" s="2">
+        <v>23.91506</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>31</v>
-      </c>
-      <c r="C14" t="s">
-        <v>32</v>
       </c>
       <c r="D14" s="4">
         <v>2021</v>
@@ -1268,13 +1300,13 @@
     </row>
     <row r="15" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" t="s">
         <v>33</v>
-      </c>
-      <c r="C15" t="s">
-        <v>34</v>
       </c>
       <c r="D15" s="4">
         <v>2021</v>
@@ -1288,13 +1320,13 @@
     </row>
     <row r="16" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" t="s">
         <v>33</v>
-      </c>
-      <c r="C16" t="s">
-        <v>34</v>
       </c>
       <c r="D16" s="4">
         <v>2024</v>
@@ -1308,13 +1340,13 @@
     </row>
     <row r="17" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" t="s">
         <v>33</v>
-      </c>
-      <c r="C17" t="s">
-        <v>34</v>
       </c>
       <c r="D17" s="4">
         <v>2035</v>
@@ -1328,13 +1360,13 @@
     </row>
     <row r="18" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D18" s="4">
         <v>2021</v>
@@ -1348,13 +1380,13 @@
     </row>
     <row r="19" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C19" t="s">
         <v>36</v>
-      </c>
-      <c r="C19" t="s">
-        <v>37</v>
       </c>
       <c r="D19" s="4">
         <v>2021</v>
@@ -1368,13 +1400,13 @@
     </row>
     <row r="20" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" t="s">
         <v>38</v>
-      </c>
-      <c r="C20" t="s">
-        <v>39</v>
       </c>
       <c r="D20" s="4">
         <v>2024</v>
@@ -1388,13 +1420,13 @@
     </row>
     <row r="21" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" t="s">
         <v>40</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>41</v>
-      </c>
-      <c r="C21" t="s">
-        <v>42</v>
       </c>
       <c r="D21" s="4">
         <v>2024</v>
@@ -1408,13 +1440,13 @@
     </row>
     <row r="22" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B22" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" t="s">
         <v>43</v>
-      </c>
-      <c r="C22" t="s">
-        <v>44</v>
       </c>
       <c r="D22" s="4">
         <v>2024</v>
@@ -1428,13 +1460,13 @@
     </row>
     <row r="23" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" t="s">
         <v>45</v>
-      </c>
-      <c r="C23" t="s">
-        <v>46</v>
       </c>
       <c r="D23" s="4">
         <v>2024</v>
@@ -1448,13 +1480,13 @@
     </row>
     <row r="24" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D24" s="4">
         <v>2024</v>
@@ -1468,10 +1500,10 @@
     </row>
     <row r="25" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C25" t="s">
         <v>8</v>
@@ -1488,13 +1520,13 @@
     </row>
     <row r="26" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B26" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" t="s">
         <v>49</v>
-      </c>
-      <c r="C26" t="s">
-        <v>50</v>
       </c>
       <c r="D26" s="4">
         <v>2024</v>
@@ -1508,13 +1540,13 @@
     </row>
     <row r="27" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D27" s="4">
         <v>2024</v>
@@ -1528,13 +1560,13 @@
     </row>
     <row r="28" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D28" s="4">
         <v>2035</v>
@@ -1548,13 +1580,13 @@
     </row>
     <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C29" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D29" s="4">
         <v>2035</v>
@@ -1568,10 +1600,10 @@
     </row>
     <row r="30" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" t="s">
         <v>53</v>
-      </c>
-      <c r="B30" t="s">
-        <v>54</v>
       </c>
       <c r="C30" t="s">
         <v>8</v>
@@ -1588,13 +1620,13 @@
     </row>
     <row r="31" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" t="s">
         <v>55</v>
-      </c>
-      <c r="C31" t="s">
-        <v>56</v>
       </c>
       <c r="D31" s="4">
         <v>2024</v>
@@ -1608,10 +1640,10 @@
     </row>
     <row r="32" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C32" t="s">
         <v>8</v>
@@ -1628,13 +1660,13 @@
     </row>
     <row r="33" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B33" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" t="s">
         <v>58</v>
-      </c>
-      <c r="C33" t="s">
-        <v>59</v>
       </c>
       <c r="D33" s="4">
         <v>2021</v>
@@ -1648,13 +1680,13 @@
     </row>
     <row r="34" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" t="s">
         <v>60</v>
-      </c>
-      <c r="C34" t="s">
-        <v>61</v>
       </c>
       <c r="D34" s="4">
         <v>2024</v>
@@ -1668,13 +1700,13 @@
     </row>
     <row r="35" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B35" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" t="s">
         <v>62</v>
-      </c>
-      <c r="C35" t="s">
-        <v>63</v>
       </c>
       <c r="D35" s="4">
         <v>2035</v>
@@ -1688,10 +1720,10 @@
     </row>
     <row r="36" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>63</v>
+      </c>
+      <c r="B36" t="s">
         <v>64</v>
-      </c>
-      <c r="B36" t="s">
-        <v>65</v>
       </c>
       <c r="C36" t="s">
         <v>8</v>
@@ -1708,13 +1740,13 @@
     </row>
     <row r="37" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" t="s">
         <v>66</v>
-      </c>
-      <c r="C37" t="s">
-        <v>67</v>
       </c>
       <c r="D37" s="4">
         <v>2035</v>
@@ -1728,10 +1760,10 @@
     </row>
     <row r="38" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" t="s">
         <v>68</v>
-      </c>
-      <c r="B38" t="s">
-        <v>69</v>
       </c>
       <c r="C38" t="s">
         <v>8</v>
@@ -1748,13 +1780,13 @@
     </row>
     <row r="39" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>69</v>
+      </c>
+      <c r="B39" t="s">
         <v>70</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>71</v>
-      </c>
-      <c r="C39" t="s">
-        <v>72</v>
       </c>
       <c r="D39" s="4">
         <v>2021</v>
@@ -1768,13 +1800,13 @@
     </row>
     <row r="40" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B40" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" t="s">
         <v>73</v>
-      </c>
-      <c r="C40" t="s">
-        <v>74</v>
       </c>
       <c r="D40" s="4">
         <v>2021</v>
@@ -1788,13 +1820,13 @@
     </row>
     <row r="41" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B41" t="s">
+        <v>74</v>
+      </c>
+      <c r="C41" t="s">
         <v>75</v>
-      </c>
-      <c r="C41" t="s">
-        <v>76</v>
       </c>
       <c r="D41" s="4">
         <v>2024</v>
@@ -1808,13 +1840,13 @@
     </row>
     <row r="42" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B42" t="s">
+        <v>76</v>
+      </c>
+      <c r="C42" t="s">
         <v>77</v>
-      </c>
-      <c r="C42" t="s">
-        <v>78</v>
       </c>
       <c r="D42" s="4">
         <v>2024</v>
@@ -1828,10 +1860,10 @@
     </row>
     <row r="43" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B43" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C43" t="s">
         <v>8</v>
@@ -1848,13 +1880,13 @@
     </row>
     <row r="44" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" t="s">
         <v>80</v>
-      </c>
-      <c r="C44" t="s">
-        <v>81</v>
       </c>
       <c r="D44" s="4">
         <v>2021</v>
@@ -1868,10 +1900,10 @@
     </row>
     <row r="45" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
+        <v>81</v>
+      </c>
+      <c r="B45" t="s">
         <v>82</v>
-      </c>
-      <c r="B45" t="s">
-        <v>83</v>
       </c>
       <c r="C45" t="s">
         <v>8</v>
@@ -1888,13 +1920,13 @@
     </row>
     <row r="46" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
+        <v>83</v>
+      </c>
+      <c r="B46" t="s">
         <v>84</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>85</v>
-      </c>
-      <c r="C46" t="s">
-        <v>86</v>
       </c>
       <c r="D46" s="4">
         <v>2021</v>
@@ -1908,10 +1940,10 @@
     </row>
     <row r="47" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>86</v>
+      </c>
+      <c r="B47" t="s">
         <v>87</v>
-      </c>
-      <c r="B47" t="s">
-        <v>88</v>
       </c>
       <c r="C47" t="s">
         <v>8</v>
@@ -1928,10 +1960,10 @@
     </row>
     <row r="48" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>88</v>
+      </c>
+      <c r="B48" t="s">
         <v>89</v>
-      </c>
-      <c r="B48" t="s">
-        <v>90</v>
       </c>
       <c r="C48" t="s">
         <v>8</v>
@@ -1948,10 +1980,10 @@
     </row>
     <row r="49" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B49" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C49" t="s">
         <v>8</v>
@@ -1963,18 +1995,18 @@
         <v>33.713389999999997</v>
       </c>
       <c r="F49" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>92</v>
+      </c>
+      <c r="B50" t="s">
         <v>93</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>94</v>
-      </c>
-      <c r="C50" t="s">
-        <v>95</v>
       </c>
       <c r="D50" s="4">
         <v>2021</v>
@@ -1988,13 +2020,13 @@
     </row>
     <row r="51" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
+        <v>92</v>
+      </c>
+      <c r="B51" t="s">
         <v>93</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
         <v>94</v>
-      </c>
-      <c r="C51" t="s">
-        <v>95</v>
       </c>
       <c r="D51" s="4">
         <v>2024</v>
@@ -2008,13 +2040,13 @@
     </row>
     <row r="52" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>92</v>
+      </c>
+      <c r="B52" t="s">
         <v>93</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>94</v>
-      </c>
-      <c r="C52" t="s">
-        <v>95</v>
       </c>
       <c r="D52" s="4">
         <v>2035</v>
@@ -2028,13 +2060,13 @@
     </row>
     <row r="53" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B53" t="s">
+        <v>95</v>
+      </c>
+      <c r="C53" t="s">
         <v>96</v>
-      </c>
-      <c r="C53" t="s">
-        <v>97</v>
       </c>
       <c r="D53" s="4">
         <v>2024</v>
@@ -2048,13 +2080,13 @@
     </row>
     <row r="54" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>97</v>
+      </c>
+      <c r="B54" t="s">
         <v>98</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>99</v>
-      </c>
-      <c r="C54" t="s">
-        <v>100</v>
       </c>
       <c r="D54" s="4">
         <v>2035</v>
@@ -2068,13 +2100,13 @@
     </row>
     <row r="55" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B55" t="s">
+        <v>100</v>
+      </c>
+      <c r="C55" t="s">
         <v>101</v>
-      </c>
-      <c r="C55" t="s">
-        <v>102</v>
       </c>
       <c r="D55" s="4">
         <v>2021</v>
@@ -2088,13 +2120,13 @@
     </row>
     <row r="56" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B56" t="s">
+        <v>100</v>
+      </c>
+      <c r="C56" t="s">
         <v>101</v>
-      </c>
-      <c r="C56" t="s">
-        <v>102</v>
       </c>
       <c r="D56" s="4">
         <v>2024</v>
@@ -2108,13 +2140,13 @@
     </row>
     <row r="57" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
+        <v>102</v>
+      </c>
+      <c r="B57" t="s">
         <v>103</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>104</v>
-      </c>
-      <c r="C57" t="s">
-        <v>105</v>
       </c>
       <c r="D57" s="4">
         <v>2021</v>
@@ -2123,15 +2155,15 @@
         <v>37.941899999999997</v>
       </c>
       <c r="F57" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
+        <v>106</v>
+      </c>
+      <c r="B58" t="s">
         <v>107</v>
-      </c>
-      <c r="B58" t="s">
-        <v>108</v>
       </c>
       <c r="C58" t="s">
         <v>8</v>
@@ -2148,13 +2180,13 @@
     </row>
     <row r="59" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
+        <v>108</v>
+      </c>
+      <c r="B59" t="s">
         <v>109</v>
       </c>
-      <c r="B59" t="s">
+      <c r="C59" t="s">
         <v>110</v>
-      </c>
-      <c r="C59" t="s">
-        <v>111</v>
       </c>
       <c r="D59" s="4">
         <v>2021</v>
@@ -2168,19 +2200,19 @@
     </row>
     <row r="60" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B60" t="s">
+        <v>111</v>
+      </c>
+      <c r="C60" t="s">
         <v>112</v>
-      </c>
-      <c r="C60" t="s">
-        <v>113</v>
       </c>
       <c r="D60" s="4">
         <v>2021</v>
       </c>
       <c r="E60" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F60" s="2">
         <v>-3.0947300000000002</v>
@@ -2188,13 +2220,13 @@
     </row>
     <row r="61" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B61" t="s">
+        <v>114</v>
+      </c>
+      <c r="C61" t="s">
         <v>115</v>
-      </c>
-      <c r="C61" t="s">
-        <v>116</v>
       </c>
       <c r="D61" s="4">
         <v>2021</v>
@@ -2208,13 +2240,13 @@
     </row>
     <row r="62" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B62" t="s">
+        <v>116</v>
+      </c>
+      <c r="C62" t="s">
         <v>117</v>
-      </c>
-      <c r="C62" t="s">
-        <v>118</v>
       </c>
       <c r="D62" s="4">
         <v>2024</v>
@@ -2228,13 +2260,13 @@
     </row>
     <row r="63" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B63" t="s">
+        <v>118</v>
+      </c>
+      <c r="C63" t="s">
         <v>119</v>
-      </c>
-      <c r="C63" t="s">
-        <v>120</v>
       </c>
       <c r="D63" s="4">
         <v>2021</v>
@@ -2248,13 +2280,13 @@
     </row>
     <row r="64" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B64" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" t="s">
         <v>121</v>
-      </c>
-      <c r="C64" t="s">
-        <v>122</v>
       </c>
       <c r="D64" s="4">
         <v>2021</v>
@@ -2268,13 +2300,13 @@
     </row>
     <row r="65" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B65" t="s">
+        <v>122</v>
+      </c>
+      <c r="C65" t="s">
         <v>123</v>
-      </c>
-      <c r="C65" t="s">
-        <v>124</v>
       </c>
       <c r="D65" s="4">
         <v>2021</v>
@@ -2288,13 +2320,13 @@
     </row>
     <row r="66" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
+        <v>124</v>
+      </c>
+      <c r="B66" t="s">
         <v>125</v>
       </c>
-      <c r="B66" t="s">
-        <v>126</v>
-      </c>
       <c r="C66" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D66" s="4">
         <v>2021</v>
@@ -2308,13 +2340,13 @@
     </row>
     <row r="67" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B67" t="s">
+        <v>126</v>
+      </c>
+      <c r="C67" t="s">
         <v>127</v>
-      </c>
-      <c r="C67" t="s">
-        <v>128</v>
       </c>
       <c r="D67" s="4">
         <v>2021</v>
@@ -2328,13 +2360,13 @@
     </row>
     <row r="68" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B68" t="s">
+        <v>128</v>
+      </c>
+      <c r="C68" t="s">
         <v>129</v>
-      </c>
-      <c r="C68" t="s">
-        <v>130</v>
       </c>
       <c r="D68" s="4">
         <v>2024</v>
@@ -2348,13 +2380,13 @@
     </row>
     <row r="69" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B69" t="s">
+        <v>130</v>
+      </c>
+      <c r="C69" t="s">
         <v>131</v>
-      </c>
-      <c r="C69" t="s">
-        <v>132</v>
       </c>
       <c r="D69" s="4">
         <v>2021</v>
@@ -2368,13 +2400,13 @@
     </row>
     <row r="70" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B70" t="s">
+        <v>132</v>
+      </c>
+      <c r="C70" t="s">
         <v>133</v>
-      </c>
-      <c r="C70" t="s">
-        <v>134</v>
       </c>
       <c r="D70" s="4">
         <v>2021</v>
@@ -2388,13 +2420,13 @@
     </row>
     <row r="71" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
+        <v>134</v>
+      </c>
+      <c r="B71" t="s">
         <v>135</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>136</v>
-      </c>
-      <c r="C71" t="s">
-        <v>137</v>
       </c>
       <c r="D71" s="4">
         <v>2021</v>
@@ -2408,13 +2440,13 @@
     </row>
     <row r="72" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
+        <v>134</v>
+      </c>
+      <c r="B72" t="s">
         <v>135</v>
       </c>
-      <c r="B72" t="s">
+      <c r="C72" t="s">
         <v>136</v>
-      </c>
-      <c r="C72" t="s">
-        <v>137</v>
       </c>
       <c r="D72" s="4">
         <v>2035</v>
@@ -2428,13 +2460,13 @@
     </row>
     <row r="73" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B73" t="s">
+        <v>137</v>
+      </c>
+      <c r="C73" t="s">
         <v>138</v>
-      </c>
-      <c r="C73" t="s">
-        <v>139</v>
       </c>
       <c r="D73" s="4">
         <v>2021</v>
@@ -2448,13 +2480,13 @@
     </row>
     <row r="74" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B74" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C74" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D74" s="4">
         <v>2021</v>
@@ -2468,13 +2500,13 @@
     </row>
     <row r="75" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B75" t="s">
+        <v>140</v>
+      </c>
+      <c r="C75" t="s">
         <v>141</v>
-      </c>
-      <c r="C75" t="s">
-        <v>142</v>
       </c>
       <c r="D75" s="4">
         <v>2021</v>
@@ -2488,13 +2520,13 @@
     </row>
     <row r="76" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
+        <v>142</v>
+      </c>
+      <c r="B76" t="s">
         <v>143</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>144</v>
-      </c>
-      <c r="C76" t="s">
-        <v>145</v>
       </c>
       <c r="D76" s="4">
         <v>2021</v>
@@ -2508,13 +2540,13 @@
     </row>
     <row r="77" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B77" t="s">
+        <v>145</v>
+      </c>
+      <c r="C77" t="s">
         <v>146</v>
-      </c>
-      <c r="C77" t="s">
-        <v>147</v>
       </c>
       <c r="D77" s="4">
         <v>2021</v>
@@ -2523,18 +2555,18 @@
         <v>59.313521000000001</v>
       </c>
       <c r="F77" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B78" t="s">
+        <v>148</v>
+      </c>
+      <c r="C78" t="s">
         <v>149</v>
-      </c>
-      <c r="C78" t="s">
-        <v>150</v>
       </c>
       <c r="D78" s="4">
         <v>2021</v>
@@ -2548,13 +2580,13 @@
     </row>
     <row r="79" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B79" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C79" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D79" s="4">
         <v>2021</v>
@@ -2568,13 +2600,13 @@
     </row>
     <row r="80" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B80" t="s">
+        <v>151</v>
+      </c>
+      <c r="C80" t="s">
         <v>152</v>
-      </c>
-      <c r="C80" t="s">
-        <v>153</v>
       </c>
       <c r="D80" s="4">
         <v>2021</v>
@@ -2612,7 +2644,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -2626,224 +2658,421 @@
     </row>
     <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C2" t="s">
-        <v>154</v>
-      </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+        <v>153</v>
+      </c>
+      <c r="D2" s="2">
+        <v>-22.911110000000001</v>
+      </c>
+      <c r="E2" s="2">
+        <v>-43.205559999999998</v>
+      </c>
     </row>
     <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C3" t="s">
         <v>156</v>
       </c>
-      <c r="B3" t="s">
-        <v>156</v>
-      </c>
-      <c r="C3" t="s">
-        <v>157</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="D3" s="2">
+        <v>29.7604267</v>
+      </c>
+      <c r="E3" s="2">
+        <v>-95.369802800000002</v>
+      </c>
     </row>
     <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B4" t="s">
+        <v>160</v>
+      </c>
+      <c r="C4" t="s">
         <v>161</v>
       </c>
-      <c r="C4" t="s">
-        <v>162</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="D4" s="2">
+        <v>4.8241699999999996</v>
+      </c>
+      <c r="E4" s="2">
+        <v>7.0336100000000004</v>
+      </c>
     </row>
     <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>162</v>
+      </c>
+      <c r="B5" t="s">
+        <v>162</v>
+      </c>
+      <c r="C5" t="s">
         <v>163</v>
       </c>
-      <c r="B5" t="s">
-        <v>163</v>
-      </c>
-      <c r="C5" t="s">
-        <v>164</v>
-      </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="D5" s="2">
+        <v>39.133330999999998</v>
+      </c>
+      <c r="E5" s="2">
+        <v>117.183334</v>
+      </c>
     </row>
     <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>164</v>
+      </c>
+      <c r="B6" t="s">
         <v>165</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>166</v>
       </c>
-      <c r="C6" t="s">
-        <v>167</v>
-      </c>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="D6" s="2">
+        <v>35.689487499999998</v>
+      </c>
+      <c r="E6" s="2">
+        <v>139.69170639999999</v>
+      </c>
     </row>
     <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" t="s">
+        <v>194</v>
+      </c>
+      <c r="C7" t="s">
         <v>168</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" s="2">
+        <v>22.466670000000001</v>
+      </c>
+      <c r="E7" s="2">
+        <v>69.066670000000002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" t="s">
+        <v>194</v>
+      </c>
+      <c r="C8" t="s">
         <v>169</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-    </row>
-    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C8" t="s">
+      <c r="D8" s="2">
+        <v>13.7563309</v>
+      </c>
+      <c r="E8" s="2">
+        <v>100.5017651</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" t="s">
         <v>170</v>
       </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-    </row>
-    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C9" t="s">
+      <c r="D9" s="2">
+        <v>28.712499999999999</v>
+      </c>
+      <c r="E9" s="2">
+        <v>33.611944000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" t="s">
+        <v>194</v>
+      </c>
+      <c r="C10" t="s">
         <v>171</v>
       </c>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
+      <c r="D10" s="2">
+        <v>31.222200000000001</v>
+      </c>
+      <c r="E10" s="2">
+        <v>121.4581</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" t="s">
+        <v>194</v>
+      </c>
+      <c r="C11" t="s">
         <v>172</v>
       </c>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
+      <c r="D11" s="2">
+        <v>38.946593999999997</v>
+      </c>
+      <c r="E11" s="2">
+        <v>121.60835299999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s">
+        <v>160</v>
+      </c>
+      <c r="C12" t="s">
         <v>173</v>
       </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C12" t="s">
+      <c r="D12" s="2">
+        <v>29.973700000000001</v>
+      </c>
+      <c r="E12" s="2">
+        <v>32.526299999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>188</v>
+      </c>
+      <c r="B13" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13" t="s">
         <v>174</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" t="s">
+      <c r="D13" s="2">
+        <v>-32.772308000000002</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-71.533302000000006</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>162</v>
+      </c>
+      <c r="B14" t="s">
+        <v>194</v>
+      </c>
+      <c r="C14" t="s">
         <v>175</v>
       </c>
-      <c r="D13" s="2"/>
-    </row>
-    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C14" t="s">
+      <c r="D14" s="2">
+        <v>22.3565</v>
+      </c>
+      <c r="E14" s="2">
+        <v>114.1362</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>189</v>
+      </c>
+      <c r="B15" t="s">
+        <v>193</v>
+      </c>
+      <c r="C15" t="s">
         <v>176</v>
       </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C15" t="s">
+      <c r="D15" s="2">
+        <v>25.285399999999999</v>
+      </c>
+      <c r="E15" s="2">
+        <v>51.530999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>190</v>
+      </c>
+      <c r="C16" t="s">
         <v>177</v>
       </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" t="s">
+      <c r="D16" s="2">
+        <v>10.183299999999999</v>
+      </c>
+      <c r="E16" s="2">
+        <v>-61.683300000000003</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>191</v>
+      </c>
+      <c r="B17" t="s">
+        <v>193</v>
+      </c>
+      <c r="C17" t="s">
         <v>178</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" t="s">
+      <c r="D17" s="2">
+        <v>25.151299999999999</v>
+      </c>
+      <c r="E17" s="2">
+        <v>52.871699999999997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B18" t="s">
+        <v>160</v>
+      </c>
+      <c r="C18" t="s">
         <v>179</v>
       </c>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C18" t="s">
+      <c r="D18" s="2">
+        <v>4.4516</v>
+      </c>
+      <c r="E18" s="2">
+        <v>7.1707400000000003</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>192</v>
+      </c>
+      <c r="B19" t="s">
+        <v>192</v>
+      </c>
+      <c r="C19" t="s">
         <v>180</v>
       </c>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C19" t="s">
+      <c r="D19" s="2">
+        <v>-12.4611</v>
+      </c>
+      <c r="E19" s="2">
+        <v>130.84200000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>160</v>
+      </c>
+      <c r="C20" t="s">
         <v>181</v>
       </c>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C20" t="s">
+      <c r="D20" s="2">
+        <v>31.2631227</v>
+      </c>
+      <c r="E20" s="2">
+        <v>32.297722</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B21" t="s">
+        <v>160</v>
+      </c>
+      <c r="C21" t="s">
         <v>182</v>
       </c>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" t="s">
+      <c r="D21" s="2">
+        <v>31.21564</v>
+      </c>
+      <c r="E21" s="2">
+        <v>29.955269999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>167</v>
+      </c>
+      <c r="B22" t="s">
+        <v>194</v>
+      </c>
+      <c r="C22" t="s">
         <v>183</v>
       </c>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C22" t="s">
+      <c r="D22" s="2">
+        <v>-1.26753</v>
+      </c>
+      <c r="E22" s="2">
+        <v>116.82899999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>106</v>
+      </c>
+      <c r="B23" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" t="s">
         <v>184</v>
       </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C23" t="s">
+      <c r="D23" s="2">
+        <v>72.102778000000001</v>
+      </c>
+      <c r="E23" s="2">
+        <v>71.25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>106</v>
+      </c>
+      <c r="B24" t="s">
+        <v>106</v>
+      </c>
+      <c r="C24" t="s">
         <v>185</v>
       </c>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C24" t="s">
-        <v>186</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D24" s="2">
+        <v>43.105600000000003</v>
+      </c>
+      <c r="E24" s="2">
+        <v>131.874</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
     </row>
-    <row r="26" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
     </row>
-    <row r="27" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
     </row>
-    <row r="28" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
-    <row r="29" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
-    <row r="30" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
     </row>
-    <row r="31" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
     </row>
-    <row r="32" spans="3:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
     </row>

</xml_diff>